<commit_message>
Refactor code structure for improved readability and maintainability; removed redundant code blocks and optimized function calls.
</commit_message>
<xml_diff>
--- a/NEWWWW1.xlsx
+++ b/NEWWWW1.xlsx
@@ -4147,6 +4147,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -4278,6 +4299,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7017,7 +7059,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -7612,6 +7654,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7743,6 +7806,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -10482,7 +10566,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -11080,6 +11164,27 @@
       <c r="AR1" t="str">
         <v/>
       </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
+      <c r="AY1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -11214,6 +11319,27 @@
       <c r="AR2" t="str">
         <v/>
       </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
+      <c r="AY2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -14007,7 +14133,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -16451,7 +16577,7 @@
         <v>18</v>
       </c>
       <c r="B22" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -31040,6 +31166,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -31171,6 +31318,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -33910,7 +34078,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -34505,6 +34673,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -34636,6 +34825,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -37375,7 +37585,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -37970,6 +38180,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -38101,6 +38332,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -40840,7 +41092,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>
@@ -41435,6 +41687,27 @@
       <c r="AQ1" t="str">
         <v/>
       </c>
+      <c r="AR1" t="str">
+        <v/>
+      </c>
+      <c r="AS1" t="str">
+        <v/>
+      </c>
+      <c r="AT1" t="str">
+        <v/>
+      </c>
+      <c r="AU1" t="str">
+        <v/>
+      </c>
+      <c r="AV1" t="str">
+        <v/>
+      </c>
+      <c r="AW1" t="str">
+        <v/>
+      </c>
+      <c r="AX1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -41566,6 +41839,27 @@
       <c r="AQ2" t="str">
         <v/>
       </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v/>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -44305,7 +44599,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MICORAL CR</v>
+        <v>MICONAZOL CR</v>
       </c>
       <c r="B21">
         <v>46874</v>

</xml_diff>